<commit_message>
frequency working, adc working, PWM_tim think it works
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32H753ZI/STM32H753ZI_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32H753ZI/STM32H753ZI_HwCfg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\fIntegration_H7\Doc\ConfigPrj\ExcelCfg\STM32H753ZI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC320765-4CCA-4C9D-ADCB-900292E39A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E59605E-7BF5-4A39-8D32-0266019849BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>

</xml_diff>